<commit_message>
Smooth labor cost to a rounded monthly amount (797,000 yen x 12)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H5mKNMdAhueiuoU89hTodu
</commit_message>
<xml_diff>
--- a/excel/Weekends_予算と報奨金_まとめ.xlsx
+++ b/excel/Weekends_予算と報奨金_まとめ.xlsx
@@ -813,12 +813,12 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>B10*12+B12+(B11*12+B12)*B13</f>
+        <f>B26*12</f>
         <v/>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>給与×12＋賞与＋法定福利</t>
+          <t>1か月分の人件費（下の行）×12</t>
         </is>
       </c>
       <c r="D21" s="2" t="n"/>
@@ -893,9 +893,20 @@
       <c r="E25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>人件費（月・1か月分に平準化）</t>
+        </is>
+      </c>
+      <c r="B26" s="11">
+        <f>ROUND((B10*12+B12+(B11*12+B12)*B13)/12,-3)</f>
+        <v/>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>（給与×12＋賞与＋法定福利）÷12を千円単位で丸めた額。賞与月も含め毎月同額で計上</t>
+        </is>
+      </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
     </row>

</xml_diff>

<commit_message>
Use annual labor cost of 9.6M yen (800k/month)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H5mKNMdAhueiuoU89hTodu
</commit_message>
<xml_diff>
--- a/excel/Weekends_予算と報奨金_まとめ.xlsx
+++ b/excel/Weekends_予算と報奨金_まとめ.xlsx
@@ -112,8 +112,8 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -789,14 +789,25 @@
       <c r="E18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>参考：人件費の積み上げ（年）</t>
+        </is>
+      </c>
+      <c r="B19" s="10">
+        <f>B10*12+B12+(B11*12+B12)*B13</f>
+        <v/>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>給与×12＋賞与＋法定福利。採用値は26行目の月額×12</t>
+        </is>
+      </c>
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>計算値</t>
         </is>
@@ -812,13 +823,13 @@
           <t>人件費（年）</t>
         </is>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="10">
         <f>B26*12</f>
         <v/>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>1か月分の人件費（下の行）×12</t>
+          <t>26行目の月額×12（年960万円）</t>
         </is>
       </c>
       <c r="D21" s="2" t="n"/>
@@ -830,7 +841,7 @@
           <t>固定費：新体制の実費（年）</t>
         </is>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="10">
         <f>B9+B8*12+B21+B14</f>
         <v/>
       </c>
@@ -848,7 +859,7 @@
           <t>固定費：本部費込み（年）</t>
         </is>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="10">
         <f>B9+B8*12+B21+B15*12</f>
         <v/>
       </c>
@@ -884,7 +895,7 @@
           <t>予算粗利（年）</t>
         </is>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="10">
         <f>B5*B6</f>
         <v/>
       </c>
@@ -898,20 +909,19 @@
           <t>人件費（月・1か月分に平準化）</t>
         </is>
       </c>
-      <c r="B26" s="11">
-        <f>ROUND((B10*12+B12+(B11*12+B12)*B13)/12,-3)</f>
-        <v/>
+      <c r="B26" s="5" t="n">
+        <v>800000</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>（給与×12＋賞与＋法定福利）÷12を千円単位で丸めた額。賞与月も含め毎月同額で計上</t>
+          <t>年960万円÷12（経営判断で指定）。賞与月も含め毎月同額で計上。参考：給与×12＋賞与＋法定福利の積み上げは下の行</t>
         </is>
       </c>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>報奨金の金額表（1人あたり月額・円）</t>
         </is>
@@ -1006,7 +1016,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>店舗合計（月）</t>
         </is>
@@ -1026,7 +1036,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>店舗合計（年・全月同じ段階）</t>
         </is>
@@ -1053,7 +1063,7 @@
       <c r="E34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>段階の判定（予算比）</t>
         </is>
@@ -1540,7 +1550,7 @@
       <c r="E18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>固定費の計</t>
         </is>
@@ -1583,7 +1593,7 @@
       <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
-      <c r="E21" s="11">
+      <c r="E21" s="10">
         <f>E19-E20</f>
         <v/>
       </c>
@@ -1698,11 +1708,11 @@
         <f>前提!B9+前提!B8*12+8091567+前提!B14</f>
         <v/>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="10">
         <f>D4*前提!$B$6</f>
         <v/>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="10">
         <f>B4/前提!$B$24</f>
         <v/>
       </c>
@@ -1714,7 +1724,7 @@
         <f>D4/前提!$B$16</f>
         <v/>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="10">
         <f>D4/12</f>
         <v/>
       </c>
@@ -1760,11 +1770,11 @@
         <f>前提!B22+前提!C33</f>
         <v/>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="10">
         <f>D6*前提!$B$6</f>
         <v/>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="10">
         <f>B6/前提!$B$24</f>
         <v/>
       </c>
@@ -1776,7 +1786,7 @@
         <f>D6/前提!$B$16</f>
         <v/>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="10">
         <f>D6/12</f>
         <v/>
       </c>
@@ -1791,11 +1801,11 @@
         <f>前提!B23</f>
         <v/>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="10">
         <f>D7*前提!$B$6</f>
         <v/>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="10">
         <f>B7/前提!$B$24</f>
         <v/>
       </c>
@@ -1807,7 +1817,7 @@
         <f>D7/前提!$B$16</f>
         <v/>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="10">
         <f>D7/12</f>
         <v/>
       </c>
@@ -1822,11 +1832,11 @@
         <f>前提!B9+前提!B8*12+10200000+前提!B15*12</f>
         <v/>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="10">
         <f>D8*前提!$B$6</f>
         <v/>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="10">
         <f>B8/前提!$B$24</f>
         <v/>
       </c>
@@ -1838,7 +1848,7 @@
         <f>D8/前提!$B$16</f>
         <v/>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="10">
         <f>D8/12</f>
         <v/>
       </c>
@@ -1892,7 +1902,7 @@
       </c>
       <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="n"/>
-      <c r="D12" s="11">
+      <c r="D12" s="10">
         <f>(0.31-前提!B7)*前提!B5-前提!B22</f>
         <v/>
       </c>
@@ -1908,7 +1918,7 @@
       </c>
       <c r="B13" s="2" t="n"/>
       <c r="C13" s="2" t="n"/>
-      <c r="D13" s="11">
+      <c r="D13" s="10">
         <f>前提!B5*0.01</f>
         <v/>
       </c>
@@ -1924,7 +1934,7 @@
       </c>
       <c r="B14" s="2" t="n"/>
       <c r="C14" s="2" t="n"/>
-      <c r="D14" s="11">
+      <c r="D14" s="10">
         <f>1000000*前提!B24</f>
         <v/>
       </c>
@@ -2062,11 +2072,11 @@
       <c r="A5" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="10">
         <f>前提!$B$5*A5</f>
         <v/>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="10">
         <f>B5*前提!$B$6</f>
         <v/>
       </c>
@@ -2074,19 +2084,19 @@
         <f>IF(A5&gt;=前提!$B$39,3,IF(A5&gt;=前提!$B$38,2,IF(A5&gt;=前提!$B$37,1,0)))</f>
         <v/>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="10">
         <f>IF(D5=0,0,INDEX(前提!$C$33:$E$33,1,D5))</f>
         <v/>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="10">
         <f>C5-B5*前提!$B$7-前提!$B$22</f>
         <v/>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="10">
         <f>F5-E5</f>
         <v/>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="10">
         <f>C5-B5*前提!$B$7-前提!$B$23-E5</f>
         <v/>
       </c>
@@ -2095,11 +2105,11 @@
       <c r="A6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="10">
         <f>前提!$B$5*A6</f>
         <v/>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="10">
         <f>B6*前提!$B$6</f>
         <v/>
       </c>
@@ -2107,19 +2117,19 @@
         <f>IF(A6&gt;=前提!$B$39,3,IF(A6&gt;=前提!$B$38,2,IF(A6&gt;=前提!$B$37,1,0)))</f>
         <v/>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="10">
         <f>IF(D6=0,0,INDEX(前提!$C$33:$E$33,1,D6))</f>
         <v/>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="10">
         <f>C6-B6*前提!$B$7-前提!$B$22</f>
         <v/>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="10">
         <f>F6-E6</f>
         <v/>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="10">
         <f>C6-B6*前提!$B$7-前提!$B$23-E6</f>
         <v/>
       </c>
@@ -2128,11 +2138,11 @@
       <c r="A7" s="6" t="n">
         <v>1.05</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="10">
         <f>前提!$B$5*A7</f>
         <v/>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="10">
         <f>B7*前提!$B$6</f>
         <v/>
       </c>
@@ -2140,19 +2150,19 @@
         <f>IF(A7&gt;=前提!$B$39,3,IF(A7&gt;=前提!$B$38,2,IF(A7&gt;=前提!$B$37,1,0)))</f>
         <v/>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="10">
         <f>IF(D7=0,0,INDEX(前提!$C$33:$E$33,1,D7))</f>
         <v/>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="10">
         <f>C7-B7*前提!$B$7-前提!$B$22</f>
         <v/>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="10">
         <f>F7-E7</f>
         <v/>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="10">
         <f>C7-B7*前提!$B$7-前提!$B$23-E7</f>
         <v/>
       </c>
@@ -2161,11 +2171,11 @@
       <c r="A8" s="6" t="n">
         <v>1.1</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="10">
         <f>前提!$B$5*A8</f>
         <v/>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="10">
         <f>B8*前提!$B$6</f>
         <v/>
       </c>
@@ -2173,19 +2183,19 @@
         <f>IF(A8&gt;=前提!$B$39,3,IF(A8&gt;=前提!$B$38,2,IF(A8&gt;=前提!$B$37,1,0)))</f>
         <v/>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="10">
         <f>IF(D8=0,0,INDEX(前提!$C$33:$E$33,1,D8))</f>
         <v/>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="10">
         <f>C8-B8*前提!$B$7-前提!$B$22</f>
         <v/>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="10">
         <f>F8-E8</f>
         <v/>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="10">
         <f>C8-B8*前提!$B$7-前提!$B$23-E8</f>
         <v/>
       </c>
@@ -2194,11 +2204,11 @@
       <c r="A9" s="6" t="n">
         <v>1.15</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="10">
         <f>前提!$B$5*A9</f>
         <v/>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="10">
         <f>B9*前提!$B$6</f>
         <v/>
       </c>
@@ -2206,19 +2216,19 @@
         <f>IF(A9&gt;=前提!$B$39,3,IF(A9&gt;=前提!$B$38,2,IF(A9&gt;=前提!$B$37,1,0)))</f>
         <v/>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="10">
         <f>IF(D9=0,0,INDEX(前提!$C$33:$E$33,1,D9))</f>
         <v/>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="10">
         <f>C9-B9*前提!$B$7-前提!$B$22</f>
         <v/>
       </c>
-      <c r="G9" s="11">
+      <c r="G9" s="10">
         <f>F9-E9</f>
         <v/>
       </c>
-      <c r="H9" s="11">
+      <c r="H9" s="10">
         <f>C9-B9*前提!$B$7-前提!$B$23-E9</f>
         <v/>
       </c>
@@ -2234,7 +2244,7 @@
       <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>粗利率だけ変えた場合（売上は予算どおり）</t>
         </is>
@@ -2277,15 +2287,15 @@
       <c r="A13" s="6" t="n">
         <v>0.31</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="10">
         <f>前提!$B$5*A13</f>
         <v/>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="10">
         <f>前提!$B$5*(A13-前提!$B$7)-前提!$B$22</f>
         <v/>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="10">
         <f>前提!$B$5*(A13-前提!$B$7)-前提!$B$23</f>
         <v/>
       </c>
@@ -2298,15 +2308,15 @@
       <c r="A14" s="6" t="n">
         <v>0.33</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="10">
         <f>前提!$B$5*A14</f>
         <v/>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="10">
         <f>前提!$B$5*(A14-前提!$B$7)-前提!$B$22</f>
         <v/>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="10">
         <f>前提!$B$5*(A14-前提!$B$7)-前提!$B$23</f>
         <v/>
       </c>
@@ -2319,15 +2329,15 @@
       <c r="A15" s="6" t="n">
         <v>0.345</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="10">
         <f>前提!$B$5*A15</f>
         <v/>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="10">
         <f>前提!$B$5*(A15-前提!$B$7)-前提!$B$22</f>
         <v/>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="10">
         <f>前提!$B$5*(A15-前提!$B$7)-前提!$B$23</f>
         <v/>
       </c>
@@ -2340,15 +2350,15 @@
       <c r="A16" s="6" t="n">
         <v>0.35</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="10">
         <f>前提!$B$5*A16</f>
         <v/>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="10">
         <f>前提!$B$5*(A16-前提!$B$7)-前提!$B$22</f>
         <v/>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="10">
         <f>前提!$B$5*(A16-前提!$B$7)-前提!$B$23</f>
         <v/>
       </c>
@@ -2361,15 +2371,15 @@
       <c r="A17" s="6" t="n">
         <v>0.36</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="10">
         <f>前提!$B$5*A17</f>
         <v/>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="10">
         <f>前提!$B$5*(A17-前提!$B$7)-前提!$B$22</f>
         <v/>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="10">
         <f>前提!$B$5*(A17-前提!$B$7)-前提!$B$23</f>
         <v/>
       </c>
@@ -2382,15 +2392,15 @@
       <c r="A18" s="6" t="n">
         <v>0.37</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="10">
         <f>前提!$B$5*A18</f>
         <v/>
       </c>
-      <c r="C18" s="11">
+      <c r="C18" s="10">
         <f>前提!$B$5*(A18-前提!$B$7)-前提!$B$22</f>
         <v/>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="10">
         <f>前提!$B$5*(A18-前提!$B$7)-前提!$B$23</f>
         <v/>
       </c>
@@ -2527,11 +2537,11 @@
           <t>2026年8月</t>
         </is>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="10">
         <f>前提!$B$5*3500000/60000000</f>
         <v/>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="10">
         <f>B4*前提!$B$6</f>
         <v/>
       </c>
@@ -2553,15 +2563,15 @@
         <f>IF(H4="","",IF(F4&lt;前提!$B$37,0,IF(H4&gt;=前提!$B$39,3,IF(H4&gt;=前提!$B$38,2,IF(H4&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J4" s="11">
+      <c r="J4" s="10">
         <f>IF(OR(I4="",I4=0),0,INDEX(前提!$C$32:$E$32,1,I4))</f>
         <v/>
       </c>
-      <c r="K4" s="11">
+      <c r="K4" s="10">
         <f>IF(E4="","",E4-D4*前提!$B$7-前提!$B$22/12-J4)</f>
         <v/>
       </c>
-      <c r="L4" s="11">
+      <c r="L4" s="10">
         <f>IF(K4="","",SUM($K$4:K4))</f>
         <v/>
       </c>
@@ -2572,11 +2582,11 @@
           <t>9月</t>
         </is>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="10">
         <f>前提!$B$5*4500000/60000000</f>
         <v/>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="10">
         <f>B5*前提!$B$6</f>
         <v/>
       </c>
@@ -2598,15 +2608,15 @@
         <f>IF(H5="","",IF(F5&lt;前提!$B$37,0,IF(H5&gt;=前提!$B$39,3,IF(H5&gt;=前提!$B$38,2,IF(H5&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="10">
         <f>IF(OR(I5="",I5=0),0,INDEX(前提!$C$32:$E$32,1,I5))</f>
         <v/>
       </c>
-      <c r="K5" s="11">
+      <c r="K5" s="10">
         <f>IF(E5="","",E5-D5*前提!$B$7-前提!$B$22/12-J5)</f>
         <v/>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="10">
         <f>IF(K5="","",SUM($K$4:K5))</f>
         <v/>
       </c>
@@ -2617,11 +2627,11 @@
           <t>10月</t>
         </is>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="10">
         <f>前提!$B$5*5500000/60000000</f>
         <v/>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="10">
         <f>B6*前提!$B$6</f>
         <v/>
       </c>
@@ -2643,15 +2653,15 @@
         <f>IF(H6="","",IF(F6&lt;前提!$B$37,0,IF(H6&gt;=前提!$B$39,3,IF(H6&gt;=前提!$B$38,2,IF(H6&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="10">
         <f>IF(OR(I6="",I6=0),0,INDEX(前提!$C$32:$E$32,1,I6))</f>
         <v/>
       </c>
-      <c r="K6" s="11">
+      <c r="K6" s="10">
         <f>IF(E6="","",E6-D6*前提!$B$7-前提!$B$22/12-J6)</f>
         <v/>
       </c>
-      <c r="L6" s="11">
+      <c r="L6" s="10">
         <f>IF(K6="","",SUM($K$4:K6))</f>
         <v/>
       </c>
@@ -2662,11 +2672,11 @@
           <t>11月</t>
         </is>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="10">
         <f>前提!$B$5*5500000/60000000</f>
         <v/>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="10">
         <f>B7*前提!$B$6</f>
         <v/>
       </c>
@@ -2688,15 +2698,15 @@
         <f>IF(H7="","",IF(F7&lt;前提!$B$37,0,IF(H7&gt;=前提!$B$39,3,IF(H7&gt;=前提!$B$38,2,IF(H7&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="10">
         <f>IF(OR(I7="",I7=0),0,INDEX(前提!$C$32:$E$32,1,I7))</f>
         <v/>
       </c>
-      <c r="K7" s="11">
+      <c r="K7" s="10">
         <f>IF(E7="","",E7-D7*前提!$B$7-前提!$B$22/12-J7)</f>
         <v/>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="10">
         <f>IF(K7="","",SUM($K$4:K7))</f>
         <v/>
       </c>
@@ -2707,11 +2717,11 @@
           <t>12月</t>
         </is>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="10">
         <f>前提!$B$5*7000000/60000000</f>
         <v/>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="10">
         <f>B8*前提!$B$6</f>
         <v/>
       </c>
@@ -2733,15 +2743,15 @@
         <f>IF(H8="","",IF(F8&lt;前提!$B$37,0,IF(H8&gt;=前提!$B$39,3,IF(H8&gt;=前提!$B$38,2,IF(H8&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="10">
         <f>IF(OR(I8="",I8=0),0,INDEX(前提!$C$32:$E$32,1,I8))</f>
         <v/>
       </c>
-      <c r="K8" s="11">
+      <c r="K8" s="10">
         <f>IF(E8="","",E8-D8*前提!$B$7-前提!$B$22/12-J8)</f>
         <v/>
       </c>
-      <c r="L8" s="11">
+      <c r="L8" s="10">
         <f>IF(K8="","",SUM($K$4:K8))</f>
         <v/>
       </c>
@@ -2752,11 +2762,11 @@
           <t>2027年1月</t>
         </is>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="10">
         <f>前提!$B$5*6000000/60000000</f>
         <v/>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="10">
         <f>B9*前提!$B$6</f>
         <v/>
       </c>
@@ -2778,15 +2788,15 @@
         <f>IF(H9="","",IF(F9&lt;前提!$B$37,0,IF(H9&gt;=前提!$B$39,3,IF(H9&gt;=前提!$B$38,2,IF(H9&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="10">
         <f>IF(OR(I9="",I9=0),0,INDEX(前提!$C$32:$E$32,1,I9))</f>
         <v/>
       </c>
-      <c r="K9" s="11">
+      <c r="K9" s="10">
         <f>IF(E9="","",E9-D9*前提!$B$7-前提!$B$22/12-J9)</f>
         <v/>
       </c>
-      <c r="L9" s="11">
+      <c r="L9" s="10">
         <f>IF(K9="","",SUM($K$4:K9))</f>
         <v/>
       </c>
@@ -2797,11 +2807,11 @@
           <t>2月</t>
         </is>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="10">
         <f>前提!$B$5*3500000/60000000</f>
         <v/>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="10">
         <f>B10*前提!$B$6</f>
         <v/>
       </c>
@@ -2823,15 +2833,15 @@
         <f>IF(H10="","",IF(F10&lt;前提!$B$37,0,IF(H10&gt;=前提!$B$39,3,IF(H10&gt;=前提!$B$38,2,IF(H10&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J10" s="11">
+      <c r="J10" s="10">
         <f>IF(OR(I10="",I10=0),0,INDEX(前提!$C$32:$E$32,1,I10))</f>
         <v/>
       </c>
-      <c r="K10" s="11">
+      <c r="K10" s="10">
         <f>IF(E10="","",E10-D10*前提!$B$7-前提!$B$22/12-J10)</f>
         <v/>
       </c>
-      <c r="L10" s="11">
+      <c r="L10" s="10">
         <f>IF(K10="","",SUM($K$4:K10))</f>
         <v/>
       </c>
@@ -2842,11 +2852,11 @@
           <t>3月</t>
         </is>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="10">
         <f>前提!$B$5*5500000/60000000</f>
         <v/>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="10">
         <f>B11*前提!$B$6</f>
         <v/>
       </c>
@@ -2868,15 +2878,15 @@
         <f>IF(H11="","",IF(F11&lt;前提!$B$37,0,IF(H11&gt;=前提!$B$39,3,IF(H11&gt;=前提!$B$38,2,IF(H11&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J11" s="11">
+      <c r="J11" s="10">
         <f>IF(OR(I11="",I11=0),0,INDEX(前提!$C$32:$E$32,1,I11))</f>
         <v/>
       </c>
-      <c r="K11" s="11">
+      <c r="K11" s="10">
         <f>IF(E11="","",E11-D11*前提!$B$7-前提!$B$22/12-J11)</f>
         <v/>
       </c>
-      <c r="L11" s="11">
+      <c r="L11" s="10">
         <f>IF(K11="","",SUM($K$4:K11))</f>
         <v/>
       </c>
@@ -2887,11 +2897,11 @@
           <t>4月</t>
         </is>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="10">
         <f>前提!$B$5*4500000/60000000</f>
         <v/>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="10">
         <f>B12*前提!$B$6</f>
         <v/>
       </c>
@@ -2913,15 +2923,15 @@
         <f>IF(H12="","",IF(F12&lt;前提!$B$37,0,IF(H12&gt;=前提!$B$39,3,IF(H12&gt;=前提!$B$38,2,IF(H12&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J12" s="11">
+      <c r="J12" s="10">
         <f>IF(OR(I12="",I12=0),0,INDEX(前提!$C$32:$E$32,1,I12))</f>
         <v/>
       </c>
-      <c r="K12" s="11">
+      <c r="K12" s="10">
         <f>IF(E12="","",E12-D12*前提!$B$7-前提!$B$22/12-J12)</f>
         <v/>
       </c>
-      <c r="L12" s="11">
+      <c r="L12" s="10">
         <f>IF(K12="","",SUM($K$4:K12))</f>
         <v/>
       </c>
@@ -2932,11 +2942,11 @@
           <t>5月</t>
         </is>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="10">
         <f>前提!$B$5*4500000/60000000</f>
         <v/>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="10">
         <f>B13*前提!$B$6</f>
         <v/>
       </c>
@@ -2958,15 +2968,15 @@
         <f>IF(H13="","",IF(F13&lt;前提!$B$37,0,IF(H13&gt;=前提!$B$39,3,IF(H13&gt;=前提!$B$38,2,IF(H13&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J13" s="11">
+      <c r="J13" s="10">
         <f>IF(OR(I13="",I13=0),0,INDEX(前提!$C$32:$E$32,1,I13))</f>
         <v/>
       </c>
-      <c r="K13" s="11">
+      <c r="K13" s="10">
         <f>IF(E13="","",E13-D13*前提!$B$7-前提!$B$22/12-J13)</f>
         <v/>
       </c>
-      <c r="L13" s="11">
+      <c r="L13" s="10">
         <f>IF(K13="","",SUM($K$4:K13))</f>
         <v/>
       </c>
@@ -2977,11 +2987,11 @@
           <t>6月</t>
         </is>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="10">
         <f>前提!$B$5*5500000/60000000</f>
         <v/>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="10">
         <f>B14*前提!$B$6</f>
         <v/>
       </c>
@@ -3003,15 +3013,15 @@
         <f>IF(H14="","",IF(F14&lt;前提!$B$37,0,IF(H14&gt;=前提!$B$39,3,IF(H14&gt;=前提!$B$38,2,IF(H14&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J14" s="11">
+      <c r="J14" s="10">
         <f>IF(OR(I14="",I14=0),0,INDEX(前提!$C$32:$E$32,1,I14))</f>
         <v/>
       </c>
-      <c r="K14" s="11">
+      <c r="K14" s="10">
         <f>IF(E14="","",E14-D14*前提!$B$7-前提!$B$22/12-J14)</f>
         <v/>
       </c>
-      <c r="L14" s="11">
+      <c r="L14" s="10">
         <f>IF(K14="","",SUM($K$4:K14))</f>
         <v/>
       </c>
@@ -3022,11 +3032,11 @@
           <t>7月</t>
         </is>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="10">
         <f>前提!$B$5*4500000/60000000</f>
         <v/>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="10">
         <f>B15*前提!$B$6</f>
         <v/>
       </c>
@@ -3048,21 +3058,21 @@
         <f>IF(H15="","",IF(F15&lt;前提!$B$37,0,IF(H15&gt;=前提!$B$39,3,IF(H15&gt;=前提!$B$38,2,IF(H15&gt;=前提!$B$37,1,0)))))</f>
         <v/>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="10">
         <f>IF(OR(I15="",I15=0),0,INDEX(前提!$C$32:$E$32,1,I15))</f>
         <v/>
       </c>
-      <c r="K15" s="11">
+      <c r="K15" s="10">
         <f>IF(E15="","",E15-D15*前提!$B$7-前提!$B$22/12-J15)</f>
         <v/>
       </c>
-      <c r="L15" s="11">
+      <c r="L15" s="10">
         <f>IF(K15="","",SUM($K$4:K15))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>年計</t>
         </is>
@@ -3175,43 +3185,43 @@
       <c r="B2" s="2" t="n"/>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>結論</t>
         </is>
       </c>
       <c r="B3" s="22" t="inlineStr">
         <is>
-          <t>予算（税抜6,000万円・粗利2,100万円）は、新体制の損益分岐（5,885万円）を2%上回るだけ。予算100%で報奨金を払うと店舗の実費はほぼトントン（+4万円）、110%で本部費込みでも黒字（+43万円）。</t>
+          <t>予算（税抜6,000万円・粗利2,100万円）は、新体制の損益分岐（5,896万円）を2%上回るだけ。予算100%で報奨金を払うと店舗の実費はちょうどトントン（+0.5万円）、110%で本部費込みでも黒字（+40万円）。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>最大の前提</t>
         </is>
       </c>
       <c r="B4" s="22" t="inlineStr">
         <is>
-          <t>粗利率35%。34.5%を切ると予算どおりでも赤字。前年並み31%なら−208万円。売上より粗利率が勝負。</t>
+          <t>粗利率35%。34.5%を切ると予算どおりでも赤字。前年並み31%なら−211万円。売上より粗利率が勝負。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>人件費</t>
         </is>
       </c>
       <c r="B5" s="22" t="inlineStr">
         <is>
-          <t>新体制は年957万円（月79.7万円）。前年実額809万円から年148万円増。回収には粗利率35%で売上約526万円の上積みが必要。</t>
+          <t>年960万円（月80万円）で計上。前年実額809万円から年151万円増。回収には粗利率35%で売上約537万円の上積みが必要。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>本部費</t>
         </is>
@@ -3223,7 +3233,7 @@
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>報奨金の設計</t>
         </is>
@@ -3235,7 +3245,7 @@
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>決めること</t>
         </is>
@@ -3247,7 +3257,7 @@
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>要確認</t>
         </is>

</xml_diff>

<commit_message>
Workbook: add monthly gross profit targets at 100% and 105% (63M plan)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H5mKNMdAhueiuoU89hTodu
</commit_message>
<xml_diff>
--- a/excel/Weekends_予算と報奨金_まとめ.xlsx
+++ b/excel/Weekends_予算と報奨金_まとめ.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="前提" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="固変分解" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="損益分岐" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="予算比シミュレーション" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="月別目標と判定" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="論点メモ" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="粗利目標（100%・105%）" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="前提" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="固変分解" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="損益分岐" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="予算比シミュレーション" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="月別目標と判定" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="論点メモ" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -492,6 +493,716 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Weekends 2027年度 月別の粗利目標（100%・105%）と報奨金</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>青字・黄色＝入力値。月の配分はスマレジの店舗予算の月比率。黄色の「実績粗利」に毎月のスマレジ粗利（税抜）を入れると段階と報奨金が出る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>年間予算売上（税抜）</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>63000000</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>社長案（売上6,300万円・粗利2,200万円・販管費2,000万円・経常利益170万円）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>年間予算粗利</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>22000000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>予算粗利率</t>
+        </is>
+      </c>
+      <c r="B6" s="12">
+        <f>B5/B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>第2段階のライン</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>報奨金 第1段階（店舗合計・月）</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>粗利が月の目標（100%）以上</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>報奨金 第2段階（店舗合計・月）</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>51000</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>粗利が月の目標の105%以上</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>予算売上</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>粗利目標 100%</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>粗利目標 105%</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>実績粗利</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>粗利 予算比</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>段階</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>報奨金（店舗計）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026年8月</t>
+        </is>
+      </c>
+      <c r="B12" s="10">
+        <f>$B$4*3500000/60000000</f>
+        <v/>
+      </c>
+      <c r="C12" s="10">
+        <f>ROUND($B$5*3500000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D12" s="10">
+        <f>ROUND(C12*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="12">
+        <f>IF(E12="","",E12/C12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="21">
+        <f>IF(E12="","",IF(E12&gt;=D12,2,IF(E12&gt;=C12,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H12" s="10">
+        <f>IF(OR(G12="",G12=0),0,IF(G12=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="B13" s="10">
+        <f>$B$4*4500000/60000000</f>
+        <v/>
+      </c>
+      <c r="C13" s="10">
+        <f>ROUND($B$5*4500000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D13" s="10">
+        <f>ROUND(C13*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="12">
+        <f>IF(E13="","",E13/C13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="21">
+        <f>IF(E13="","",IF(E13&gt;=D13,2,IF(E13&gt;=C13,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H13" s="10">
+        <f>IF(OR(G13="",G13=0),0,IF(G13=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>10月</t>
+        </is>
+      </c>
+      <c r="B14" s="10">
+        <f>$B$4*5500000/60000000</f>
+        <v/>
+      </c>
+      <c r="C14" s="10">
+        <f>ROUND($B$5*5500000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D14" s="10">
+        <f>ROUND(C14*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="12">
+        <f>IF(E14="","",E14/C14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>IF(E14="","",IF(E14&gt;=D14,2,IF(E14&gt;=C14,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H14" s="10">
+        <f>IF(OR(G14="",G14=0),0,IF(G14=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="B15" s="10">
+        <f>$B$4*5500000/60000000</f>
+        <v/>
+      </c>
+      <c r="C15" s="10">
+        <f>ROUND($B$5*5500000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D15" s="10">
+        <f>ROUND(C15*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="12">
+        <f>IF(E15="","",E15/C15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="21">
+        <f>IF(E15="","",IF(E15&gt;=D15,2,IF(E15&gt;=C15,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H15" s="10">
+        <f>IF(OR(G15="",G15=0),0,IF(G15=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="B16" s="10">
+        <f>$B$4*7000000/60000000</f>
+        <v/>
+      </c>
+      <c r="C16" s="10">
+        <f>ROUND($B$5*7000000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D16" s="10">
+        <f>ROUND(C16*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="12">
+        <f>IF(E16="","",E16/C16)</f>
+        <v/>
+      </c>
+      <c r="G16" s="21">
+        <f>IF(E16="","",IF(E16&gt;=D16,2,IF(E16&gt;=C16,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H16" s="10">
+        <f>IF(OR(G16="",G16=0),0,IF(G16=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>2027年1月</t>
+        </is>
+      </c>
+      <c r="B17" s="10">
+        <f>$B$4*6000000/60000000</f>
+        <v/>
+      </c>
+      <c r="C17" s="10">
+        <f>ROUND($B$5*6000000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D17" s="10">
+        <f>ROUND(C17*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="12">
+        <f>IF(E17="","",E17/C17)</f>
+        <v/>
+      </c>
+      <c r="G17" s="21">
+        <f>IF(E17="","",IF(E17&gt;=D17,2,IF(E17&gt;=C17,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H17" s="10">
+        <f>IF(OR(G17="",G17=0),0,IF(G17=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2月</t>
+        </is>
+      </c>
+      <c r="B18" s="10">
+        <f>$B$4*3500000/60000000</f>
+        <v/>
+      </c>
+      <c r="C18" s="10">
+        <f>ROUND($B$5*3500000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D18" s="10">
+        <f>ROUND(C18*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="12">
+        <f>IF(E18="","",E18/C18)</f>
+        <v/>
+      </c>
+      <c r="G18" s="21">
+        <f>IF(E18="","",IF(E18&gt;=D18,2,IF(E18&gt;=C18,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H18" s="10">
+        <f>IF(OR(G18="",G18=0),0,IF(G18=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>3月</t>
+        </is>
+      </c>
+      <c r="B19" s="10">
+        <f>$B$4*5500000/60000000</f>
+        <v/>
+      </c>
+      <c r="C19" s="10">
+        <f>ROUND($B$5*5500000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D19" s="10">
+        <f>ROUND(C19*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="12">
+        <f>IF(E19="","",E19/C19)</f>
+        <v/>
+      </c>
+      <c r="G19" s="21">
+        <f>IF(E19="","",IF(E19&gt;=D19,2,IF(E19&gt;=C19,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H19" s="10">
+        <f>IF(OR(G19="",G19=0),0,IF(G19=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>4月</t>
+        </is>
+      </c>
+      <c r="B20" s="10">
+        <f>$B$4*4500000/60000000</f>
+        <v/>
+      </c>
+      <c r="C20" s="10">
+        <f>ROUND($B$5*4500000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D20" s="10">
+        <f>ROUND(C20*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="12">
+        <f>IF(E20="","",E20/C20)</f>
+        <v/>
+      </c>
+      <c r="G20" s="21">
+        <f>IF(E20="","",IF(E20&gt;=D20,2,IF(E20&gt;=C20,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H20" s="10">
+        <f>IF(OR(G20="",G20=0),0,IF(G20=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="B21" s="10">
+        <f>$B$4*4500000/60000000</f>
+        <v/>
+      </c>
+      <c r="C21" s="10">
+        <f>ROUND($B$5*4500000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D21" s="10">
+        <f>ROUND(C21*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="12">
+        <f>IF(E21="","",E21/C21)</f>
+        <v/>
+      </c>
+      <c r="G21" s="21">
+        <f>IF(E21="","",IF(E21&gt;=D21,2,IF(E21&gt;=C21,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H21" s="10">
+        <f>IF(OR(G21="",G21=0),0,IF(G21=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="B22" s="10">
+        <f>$B$4*5500000/60000000</f>
+        <v/>
+      </c>
+      <c r="C22" s="10">
+        <f>ROUND($B$5*5500000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D22" s="10">
+        <f>ROUND(C22*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="12">
+        <f>IF(E22="","",E22/C22)</f>
+        <v/>
+      </c>
+      <c r="G22" s="21">
+        <f>IF(E22="","",IF(E22&gt;=D22,2,IF(E22&gt;=C22,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H22" s="10">
+        <f>IF(OR(G22="",G22=0),0,IF(G22=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>7月</t>
+        </is>
+      </c>
+      <c r="B23" s="10">
+        <f>$B$4*4500000/60000000</f>
+        <v/>
+      </c>
+      <c r="C23" s="10">
+        <f>ROUND($B$5*4500000/60000000,-3)</f>
+        <v/>
+      </c>
+      <c r="D23" s="10">
+        <f>ROUND(C23*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="12">
+        <f>IF(E23="","",E23/C23)</f>
+        <v/>
+      </c>
+      <c r="G23" s="21">
+        <f>IF(E23="","",IF(E23&gt;=D23,2,IF(E23&gt;=C23,1,0)))</f>
+        <v/>
+      </c>
+      <c r="H23" s="10">
+        <f>IF(OR(G23="",G23=0),0,IF(G23=2,$B$9,$B$8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>年計</t>
+        </is>
+      </c>
+      <c r="B24" s="14">
+        <f>SUM(B12:B23)</f>
+        <v/>
+      </c>
+      <c r="C24" s="14">
+        <f>SUM(C12:C23)</f>
+        <v/>
+      </c>
+      <c r="D24" s="14">
+        <f>SUM(D12:D23)</f>
+        <v/>
+      </c>
+      <c r="E24" s="14">
+        <f>SUM(E12:E23)</f>
+        <v/>
+      </c>
+      <c r="H24" s="14">
+        <f>SUM(H12:H23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>全月達成した場合の報奨金（年）</t>
+        </is>
+      </c>
+      <c r="C25" s="14">
+        <f>B8*12</f>
+        <v/>
+      </c>
+      <c r="D25" s="14">
+        <f>B9*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>1人あたりの月額（店舗計を配分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>区分</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>人数</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>配分の重み</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>第1段階（円）</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>第2段階（円）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>店長</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="D29" s="10">
+        <f>ROUND($B$8*C29/SUMPRODUCT($B$29:$B$31,$C$29:$C$31),-2)</f>
+        <v/>
+      </c>
+      <c r="E29" s="10">
+        <f>ROUND($B$9*C29/SUMPRODUCT($B$29:$B$31,$C$29:$C$31),-2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>古参パート</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="D30" s="10">
+        <f>ROUND($B$8*C30/SUMPRODUCT($B$29:$B$31,$C$29:$C$31),-2)</f>
+        <v/>
+      </c>
+      <c r="E30" s="10">
+        <f>ROUND($B$9*C30/SUMPRODUCT($B$29:$B$31,$C$29:$C$31),-2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>その他パート</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="D31" s="10">
+        <f>ROUND($B$8*C31/SUMPRODUCT($B$29:$B$31,$C$29:$C$31),-2)</f>
+        <v/>
+      </c>
+      <c r="E31" s="10">
+        <f>ROUND($B$9*C31/SUMPRODUCT($B$29:$B$31,$C$29:$C$31),-2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>合計（月）</t>
+        </is>
+      </c>
+      <c r="D32" s="14">
+        <f>SUMPRODUCT(B29:B31,D29:D31)</f>
+        <v/>
+      </c>
+      <c r="E32" s="14">
+        <f>SUMPRODUCT(B29:B31,E29:E31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>考え方：第1段階（月3万円・年36万円）は予算達成時の経常利益の約半分。第2段階は、105%達成で増える利益（年約88万円）の約3割を上乗せした額（月5.1万円・年61万円）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>判定は粗利額のみ（売上は参考）。粗利目標は千円単位で丸め。処分品は粗利の計算から除く。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1155,7 +1866,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1621,7 +2332,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1969,7 +2680,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2414,7 +3125,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3159,7 +3870,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Workbook: monthly GP targets by prior-year composition and Smaregi ratio
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H5mKNMdAhueiuoU89hTodu
</commit_message>
<xml_diff>
--- a/excel/Weekends_予算と報奨金_まとめ.xlsx
+++ b/excel/Weekends_予算と報奨金_まとめ.xlsx
@@ -100,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,6 +128,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -493,19 +495,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,7 +523,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>青字・黄色＝入力値。月の配分はスマレジの店舗予算の月比率。黄色の「実績粗利」に毎月のスマレジ粗利（税抜）を入れると段階と報奨金が出る。</t>
+          <t>青字・黄色＝入力値。月の目標は「前年の売上構成比」版と「スマレジ予算の月比率」版の2つ。B10で判定に使う版を選び、黄色の「実績粗利」にスマレジ粗利（税抜）を入れると段階と報奨金が出る。</t>
         </is>
       </c>
     </row>
@@ -598,6 +603,16 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>判定に使う目標（1=前年構成比版、2=スマレジ版）</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="n">
+        <v>1</v>
+      </c>
+    </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -606,35 +621,60 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>予算売上</t>
+          <t>前年売上（参考）</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>粗利目標 100%</t>
+          <t>前年構成比</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>粗利目標 105%</t>
+          <t>目標売上（参考）</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
+          <t>粗利目標100%（構成比版）</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>粗利目標105%（構成比版）</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>粗利目標100%（スマレジ版）</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>粗利目標105%（スマレジ版）</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
           <t>実績粗利</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>判定に使う100%目標</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>粗利 予算比</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>段階</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>報奨金（店舗計）</t>
         </is>
@@ -646,29 +686,48 @@
           <t>2026年8月</t>
         </is>
       </c>
-      <c r="B12" s="10">
-        <f>$B$4*3500000/60000000</f>
-        <v/>
-      </c>
-      <c r="C12" s="10">
+      <c r="B12" s="8" t="n">
+        <v>3040292</v>
+      </c>
+      <c r="C12" s="12">
+        <f>B12/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D12" s="10">
+        <f>ROUND($B$4*C12,-3)</f>
+        <v/>
+      </c>
+      <c r="E12" s="10">
+        <f>ROUND($B$5*C12,-3)</f>
+        <v/>
+      </c>
+      <c r="F12" s="10">
+        <f>ROUND(E12*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G12" s="10">
         <f>ROUND($B$5*3500000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D12" s="10">
-        <f>ROUND(C12*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="12">
-        <f>IF(E12="","",E12/C12)</f>
-        <v/>
-      </c>
-      <c r="G12" s="21">
-        <f>IF(E12="","",IF(E12&gt;=D12,2,IF(E12&gt;=C12,1,0)))</f>
-        <v/>
-      </c>
       <c r="H12" s="10">
-        <f>IF(OR(G12="",G12=0),0,IF(G12=2,$B$9,$B$8))</f>
+        <f>ROUND(G12*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="10">
+        <f>IF($B$10=2,G12,E12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="12">
+        <f>IF(I12="","",I12/J12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="21">
+        <f>IF(I12="","",IF(I12&gt;=ROUND(J12*$B$7,-3),2,IF(I12&gt;=J12,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M12" s="10">
+        <f>IF(OR(L12="",L12=0),0,IF(L12=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -678,29 +737,48 @@
           <t>9月</t>
         </is>
       </c>
-      <c r="B13" s="10">
-        <f>$B$4*4500000/60000000</f>
-        <v/>
-      </c>
-      <c r="C13" s="10">
+      <c r="B13" s="8" t="n">
+        <v>3638478</v>
+      </c>
+      <c r="C13" s="12">
+        <f>B13/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D13" s="10">
+        <f>ROUND($B$4*C13,-3)</f>
+        <v/>
+      </c>
+      <c r="E13" s="10">
+        <f>ROUND($B$5*C13,-3)</f>
+        <v/>
+      </c>
+      <c r="F13" s="10">
+        <f>ROUND(E13*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G13" s="10">
         <f>ROUND($B$5*4500000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D13" s="10">
-        <f>ROUND(C13*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="12">
-        <f>IF(E13="","",E13/C13)</f>
-        <v/>
-      </c>
-      <c r="G13" s="21">
-        <f>IF(E13="","",IF(E13&gt;=D13,2,IF(E13&gt;=C13,1,0)))</f>
-        <v/>
-      </c>
       <c r="H13" s="10">
-        <f>IF(OR(G13="",G13=0),0,IF(G13=2,$B$9,$B$8))</f>
+        <f>ROUND(G13*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="10">
+        <f>IF($B$10=2,G13,E13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="12">
+        <f>IF(I13="","",I13/J13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="21">
+        <f>IF(I13="","",IF(I13&gt;=ROUND(J13*$B$7,-3),2,IF(I13&gt;=J13,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M13" s="10">
+        <f>IF(OR(L13="",L13=0),0,IF(L13=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -710,29 +788,48 @@
           <t>10月</t>
         </is>
       </c>
-      <c r="B14" s="10">
-        <f>$B$4*5500000/60000000</f>
-        <v/>
-      </c>
-      <c r="C14" s="10">
+      <c r="B14" s="8" t="n">
+        <v>4934704</v>
+      </c>
+      <c r="C14" s="12">
+        <f>B14/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D14" s="10">
+        <f>ROUND($B$4*C14,-3)</f>
+        <v/>
+      </c>
+      <c r="E14" s="10">
+        <f>ROUND($B$5*C14,-3)</f>
+        <v/>
+      </c>
+      <c r="F14" s="10">
+        <f>ROUND(E14*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G14" s="10">
         <f>ROUND($B$5*5500000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D14" s="10">
-        <f>ROUND(C14*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="12">
-        <f>IF(E14="","",E14/C14)</f>
-        <v/>
-      </c>
-      <c r="G14" s="21">
-        <f>IF(E14="","",IF(E14&gt;=D14,2,IF(E14&gt;=C14,1,0)))</f>
-        <v/>
-      </c>
       <c r="H14" s="10">
-        <f>IF(OR(G14="",G14=0),0,IF(G14=2,$B$9,$B$8))</f>
+        <f>ROUND(G14*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="10">
+        <f>IF($B$10=2,G14,E14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="12">
+        <f>IF(I14="","",I14/J14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="21">
+        <f>IF(I14="","",IF(I14&gt;=ROUND(J14*$B$7,-3),2,IF(I14&gt;=J14,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M14" s="10">
+        <f>IF(OR(L14="",L14=0),0,IF(L14=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -742,29 +839,48 @@
           <t>11月</t>
         </is>
       </c>
-      <c r="B15" s="10">
-        <f>$B$4*5500000/60000000</f>
-        <v/>
-      </c>
-      <c r="C15" s="10">
+      <c r="B15" s="8" t="n">
+        <v>5149749</v>
+      </c>
+      <c r="C15" s="12">
+        <f>B15/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D15" s="10">
+        <f>ROUND($B$4*C15,-3)</f>
+        <v/>
+      </c>
+      <c r="E15" s="10">
+        <f>ROUND($B$5*C15,-3)</f>
+        <v/>
+      </c>
+      <c r="F15" s="10">
+        <f>ROUND(E15*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G15" s="10">
         <f>ROUND($B$5*5500000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D15" s="10">
-        <f>ROUND(C15*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="12">
-        <f>IF(E15="","",E15/C15)</f>
-        <v/>
-      </c>
-      <c r="G15" s="21">
-        <f>IF(E15="","",IF(E15&gt;=D15,2,IF(E15&gt;=C15,1,0)))</f>
-        <v/>
-      </c>
       <c r="H15" s="10">
-        <f>IF(OR(G15="",G15=0),0,IF(G15=2,$B$9,$B$8))</f>
+        <f>ROUND(G15*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="10">
+        <f>IF($B$10=2,G15,E15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="12">
+        <f>IF(I15="","",I15/J15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="21">
+        <f>IF(I15="","",IF(I15&gt;=ROUND(J15*$B$7,-3),2,IF(I15&gt;=J15,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M15" s="10">
+        <f>IF(OR(L15="",L15=0),0,IF(L15=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -774,29 +890,48 @@
           <t>12月</t>
         </is>
       </c>
-      <c r="B16" s="10">
-        <f>$B$4*7000000/60000000</f>
-        <v/>
-      </c>
-      <c r="C16" s="10">
+      <c r="B16" s="8" t="n">
+        <v>6820952</v>
+      </c>
+      <c r="C16" s="12">
+        <f>B16/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D16" s="10">
+        <f>ROUND($B$4*C16,-3)</f>
+        <v/>
+      </c>
+      <c r="E16" s="10">
+        <f>ROUND($B$5*C16,-3)</f>
+        <v/>
+      </c>
+      <c r="F16" s="10">
+        <f>ROUND(E16*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G16" s="10">
         <f>ROUND($B$5*7000000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D16" s="10">
-        <f>ROUND(C16*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="12">
-        <f>IF(E16="","",E16/C16)</f>
-        <v/>
-      </c>
-      <c r="G16" s="21">
-        <f>IF(E16="","",IF(E16&gt;=D16,2,IF(E16&gt;=C16,1,0)))</f>
-        <v/>
-      </c>
       <c r="H16" s="10">
-        <f>IF(OR(G16="",G16=0),0,IF(G16=2,$B$9,$B$8))</f>
+        <f>ROUND(G16*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="10">
+        <f>IF($B$10=2,G16,E16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="12">
+        <f>IF(I16="","",I16/J16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="21">
+        <f>IF(I16="","",IF(I16&gt;=ROUND(J16*$B$7,-3),2,IF(I16&gt;=J16,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M16" s="10">
+        <f>IF(OR(L16="",L16=0),0,IF(L16=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -806,29 +941,48 @@
           <t>2027年1月</t>
         </is>
       </c>
-      <c r="B17" s="10">
-        <f>$B$4*6000000/60000000</f>
-        <v/>
-      </c>
-      <c r="C17" s="10">
+      <c r="B17" s="8" t="n">
+        <v>4850701</v>
+      </c>
+      <c r="C17" s="12">
+        <f>B17/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D17" s="10">
+        <f>ROUND($B$4*C17,-3)</f>
+        <v/>
+      </c>
+      <c r="E17" s="10">
+        <f>ROUND($B$5*C17,-3)</f>
+        <v/>
+      </c>
+      <c r="F17" s="10">
+        <f>ROUND(E17*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G17" s="10">
         <f>ROUND($B$5*6000000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D17" s="10">
-        <f>ROUND(C17*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="12">
-        <f>IF(E17="","",E17/C17)</f>
-        <v/>
-      </c>
-      <c r="G17" s="21">
-        <f>IF(E17="","",IF(E17&gt;=D17,2,IF(E17&gt;=C17,1,0)))</f>
-        <v/>
-      </c>
       <c r="H17" s="10">
-        <f>IF(OR(G17="",G17=0),0,IF(G17=2,$B$9,$B$8))</f>
+        <f>ROUND(G17*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="10">
+        <f>IF($B$10=2,G17,E17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="12">
+        <f>IF(I17="","",I17/J17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="21">
+        <f>IF(I17="","",IF(I17&gt;=ROUND(J17*$B$7,-3),2,IF(I17&gt;=J17,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M17" s="10">
+        <f>IF(OR(L17="",L17=0),0,IF(L17=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -838,29 +992,48 @@
           <t>2月</t>
         </is>
       </c>
-      <c r="B18" s="10">
-        <f>$B$4*3500000/60000000</f>
-        <v/>
-      </c>
-      <c r="C18" s="10">
+      <c r="B18" s="8" t="n">
+        <v>2795656</v>
+      </c>
+      <c r="C18" s="12">
+        <f>B18/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D18" s="10">
+        <f>ROUND($B$4*C18,-3)</f>
+        <v/>
+      </c>
+      <c r="E18" s="10">
+        <f>ROUND($B$5*C18,-3)</f>
+        <v/>
+      </c>
+      <c r="F18" s="10">
+        <f>ROUND(E18*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G18" s="10">
         <f>ROUND($B$5*3500000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D18" s="10">
-        <f>ROUND(C18*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="12">
-        <f>IF(E18="","",E18/C18)</f>
-        <v/>
-      </c>
-      <c r="G18" s="21">
-        <f>IF(E18="","",IF(E18&gt;=D18,2,IF(E18&gt;=C18,1,0)))</f>
-        <v/>
-      </c>
       <c r="H18" s="10">
-        <f>IF(OR(G18="",G18=0),0,IF(G18=2,$B$9,$B$8))</f>
+        <f>ROUND(G18*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="10">
+        <f>IF($B$10=2,G18,E18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="12">
+        <f>IF(I18="","",I18/J18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="21">
+        <f>IF(I18="","",IF(I18&gt;=ROUND(J18*$B$7,-3),2,IF(I18&gt;=J18,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M18" s="10">
+        <f>IF(OR(L18="",L18=0),0,IF(L18=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -870,29 +1043,48 @@
           <t>3月</t>
         </is>
       </c>
-      <c r="B19" s="10">
-        <f>$B$4*5500000/60000000</f>
-        <v/>
-      </c>
-      <c r="C19" s="10">
+      <c r="B19" s="8" t="n">
+        <v>4419804</v>
+      </c>
+      <c r="C19" s="12">
+        <f>B19/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D19" s="10">
+        <f>ROUND($B$4*C19,-3)</f>
+        <v/>
+      </c>
+      <c r="E19" s="10">
+        <f>ROUND($B$5*C19,-3)</f>
+        <v/>
+      </c>
+      <c r="F19" s="10">
+        <f>ROUND(E19*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G19" s="10">
         <f>ROUND($B$5*5500000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D19" s="10">
-        <f>ROUND(C19*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="12">
-        <f>IF(E19="","",E19/C19)</f>
-        <v/>
-      </c>
-      <c r="G19" s="21">
-        <f>IF(E19="","",IF(E19&gt;=D19,2,IF(E19&gt;=C19,1,0)))</f>
-        <v/>
-      </c>
       <c r="H19" s="10">
-        <f>IF(OR(G19="",G19=0),0,IF(G19=2,$B$9,$B$8))</f>
+        <f>ROUND(G19*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I19" s="5" t="n"/>
+      <c r="J19" s="10">
+        <f>IF($B$10=2,G19,E19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="12">
+        <f>IF(I19="","",I19/J19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="21">
+        <f>IF(I19="","",IF(I19&gt;=ROUND(J19*$B$7,-3),2,IF(I19&gt;=J19,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M19" s="10">
+        <f>IF(OR(L19="",L19=0),0,IF(L19=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -902,29 +1094,48 @@
           <t>4月</t>
         </is>
       </c>
-      <c r="B20" s="10">
-        <f>$B$4*4500000/60000000</f>
-        <v/>
-      </c>
-      <c r="C20" s="10">
+      <c r="B20" s="8" t="n">
+        <v>3581469</v>
+      </c>
+      <c r="C20" s="12">
+        <f>B20/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D20" s="10">
+        <f>ROUND($B$4*C20,-3)</f>
+        <v/>
+      </c>
+      <c r="E20" s="10">
+        <f>ROUND($B$5*C20,-3)</f>
+        <v/>
+      </c>
+      <c r="F20" s="10">
+        <f>ROUND(E20*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G20" s="10">
         <f>ROUND($B$5*4500000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D20" s="10">
-        <f>ROUND(C20*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="12">
-        <f>IF(E20="","",E20/C20)</f>
-        <v/>
-      </c>
-      <c r="G20" s="21">
-        <f>IF(E20="","",IF(E20&gt;=D20,2,IF(E20&gt;=C20,1,0)))</f>
-        <v/>
-      </c>
       <c r="H20" s="10">
-        <f>IF(OR(G20="",G20=0),0,IF(G20=2,$B$9,$B$8))</f>
+        <f>ROUND(G20*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I20" s="5" t="n"/>
+      <c r="J20" s="10">
+        <f>IF($B$10=2,G20,E20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="12">
+        <f>IF(I20="","",I20/J20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="21">
+        <f>IF(I20="","",IF(I20&gt;=ROUND(J20*$B$7,-3),2,IF(I20&gt;=J20,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M20" s="10">
+        <f>IF(OR(L20="",L20=0),0,IF(L20=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -934,29 +1145,48 @@
           <t>5月</t>
         </is>
       </c>
-      <c r="B21" s="10">
-        <f>$B$4*4500000/60000000</f>
-        <v/>
-      </c>
-      <c r="C21" s="10">
+      <c r="B21" s="8" t="n">
+        <v>4799124</v>
+      </c>
+      <c r="C21" s="12">
+        <f>B21/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D21" s="10">
+        <f>ROUND($B$4*C21,-3)</f>
+        <v/>
+      </c>
+      <c r="E21" s="10">
+        <f>ROUND($B$5*C21,-3)</f>
+        <v/>
+      </c>
+      <c r="F21" s="10">
+        <f>ROUND(E21*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G21" s="10">
         <f>ROUND($B$5*4500000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D21" s="10">
-        <f>ROUND(C21*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="12">
-        <f>IF(E21="","",E21/C21)</f>
-        <v/>
-      </c>
-      <c r="G21" s="21">
-        <f>IF(E21="","",IF(E21&gt;=D21,2,IF(E21&gt;=C21,1,0)))</f>
-        <v/>
-      </c>
       <c r="H21" s="10">
-        <f>IF(OR(G21="",G21=0),0,IF(G21=2,$B$9,$B$8))</f>
+        <f>ROUND(G21*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I21" s="5" t="n"/>
+      <c r="J21" s="10">
+        <f>IF($B$10=2,G21,E21)</f>
+        <v/>
+      </c>
+      <c r="K21" s="12">
+        <f>IF(I21="","",I21/J21)</f>
+        <v/>
+      </c>
+      <c r="L21" s="21">
+        <f>IF(I21="","",IF(I21&gt;=ROUND(J21*$B$7,-3),2,IF(I21&gt;=J21,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M21" s="10">
+        <f>IF(OR(L21="",L21=0),0,IF(L21=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -966,29 +1196,48 @@
           <t>6月</t>
         </is>
       </c>
-      <c r="B22" s="10">
-        <f>$B$4*5500000/60000000</f>
-        <v/>
-      </c>
-      <c r="C22" s="10">
+      <c r="B22" s="8" t="n">
+        <v>4888307</v>
+      </c>
+      <c r="C22" s="12">
+        <f>B22/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D22" s="10">
+        <f>ROUND($B$4*C22,-3)</f>
+        <v/>
+      </c>
+      <c r="E22" s="10">
+        <f>ROUND($B$5*C22,-3)</f>
+        <v/>
+      </c>
+      <c r="F22" s="10">
+        <f>ROUND(E22*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G22" s="10">
         <f>ROUND($B$5*5500000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D22" s="10">
-        <f>ROUND(C22*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="12">
-        <f>IF(E22="","",E22/C22)</f>
-        <v/>
-      </c>
-      <c r="G22" s="21">
-        <f>IF(E22="","",IF(E22&gt;=D22,2,IF(E22&gt;=C22,1,0)))</f>
-        <v/>
-      </c>
       <c r="H22" s="10">
-        <f>IF(OR(G22="",G22=0),0,IF(G22=2,$B$9,$B$8))</f>
+        <f>ROUND(G22*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I22" s="5" t="n"/>
+      <c r="J22" s="10">
+        <f>IF($B$10=2,G22,E22)</f>
+        <v/>
+      </c>
+      <c r="K22" s="12">
+        <f>IF(I22="","",I22/J22)</f>
+        <v/>
+      </c>
+      <c r="L22" s="21">
+        <f>IF(I22="","",IF(I22&gt;=ROUND(J22*$B$7,-3),2,IF(I22&gt;=J22,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M22" s="10">
+        <f>IF(OR(L22="",L22=0),0,IF(L22=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -998,29 +1247,48 @@
           <t>7月</t>
         </is>
       </c>
-      <c r="B23" s="10">
-        <f>$B$4*4500000/60000000</f>
-        <v/>
-      </c>
-      <c r="C23" s="10">
+      <c r="B23" s="8" t="n">
+        <v>4741065</v>
+      </c>
+      <c r="C23" s="12">
+        <f>B23/SUM($B$12:$B$23)</f>
+        <v/>
+      </c>
+      <c r="D23" s="10">
+        <f>ROUND($B$4*C23,-3)</f>
+        <v/>
+      </c>
+      <c r="E23" s="10">
+        <f>ROUND($B$5*C23,-3)</f>
+        <v/>
+      </c>
+      <c r="F23" s="10">
+        <f>ROUND(E23*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="G23" s="10">
         <f>ROUND($B$5*4500000/60000000,-3)</f>
         <v/>
       </c>
-      <c r="D23" s="10">
-        <f>ROUND(C23*$B$7,-3)</f>
-        <v/>
-      </c>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="12">
-        <f>IF(E23="","",E23/C23)</f>
-        <v/>
-      </c>
-      <c r="G23" s="21">
-        <f>IF(E23="","",IF(E23&gt;=D23,2,IF(E23&gt;=C23,1,0)))</f>
-        <v/>
-      </c>
       <c r="H23" s="10">
-        <f>IF(OR(G23="",G23=0),0,IF(G23=2,$B$9,$B$8))</f>
+        <f>ROUND(G23*$B$7,-3)</f>
+        <v/>
+      </c>
+      <c r="I23" s="5" t="n"/>
+      <c r="J23" s="10">
+        <f>IF($B$10=2,G23,E23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="12">
+        <f>IF(I23="","",I23/J23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="21">
+        <f>IF(I23="","",IF(I23&gt;=ROUND(J23*$B$7,-3),2,IF(I23&gt;=J23,1,0)))</f>
+        <v/>
+      </c>
+      <c r="M23" s="10">
+        <f>IF(OR(L23="",L23=0),0,IF(L23=2,$B$9,$B$8))</f>
         <v/>
       </c>
     </row>
@@ -1034,7 +1302,7 @@
         <f>SUM(B12:B23)</f>
         <v/>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="24">
         <f>SUM(C12:C23)</f>
         <v/>
       </c>
@@ -1046,10 +1314,30 @@
         <f>SUM(E12:E23)</f>
         <v/>
       </c>
+      <c r="F24" s="14">
+        <f>SUM(F12:F23)</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>SUM(G12:G23)</f>
+        <v/>
+      </c>
       <c r="H24" s="14">
         <f>SUM(H12:H23)</f>
         <v/>
       </c>
+      <c r="I24" s="14">
+        <f>SUM(I12:I23)</f>
+        <v/>
+      </c>
+      <c r="J24" s="14">
+        <f>SUM(J12:J23)</f>
+        <v/>
+      </c>
+      <c r="M24" s="14">
+        <f>SUM(M12:M23)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -1057,13 +1345,20 @@
           <t>全月達成した場合の報奨金（年）</t>
         </is>
       </c>
-      <c r="C25" s="14">
+      <c r="E25" s="14">
         <f>B8*12</f>
         <v/>
       </c>
-      <c r="D25" s="14">
+      <c r="F25" s="14">
         <f>B9*12</f>
         <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>前年構成比＝2025/8〜2026/7の月別売上（発展会計）の比率。会計の月次粗利は棚卸の調整で振れる（1月−124万円）ため、配分には売上の比率を使う。千円単位の丸めで年計が±1千円ずれることがある。</t>
+        </is>
       </c>
     </row>
     <row r="27">

</xml_diff>

<commit_message>
Workbook: GP target 21.5M at 35% with incentive tiers 30k/50k
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H5mKNMdAhueiuoU89hTodu
</commit_message>
<xml_diff>
--- a/excel/Weekends_予算と報奨金_まとめ.xlsx
+++ b/excel/Weekends_予算と報奨金_まとめ.xlsx
@@ -533,23 +533,24 @@
           <t>年間予算売上（税抜）</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
-        <v>63000000</v>
+      <c r="B4" s="10">
+        <f>ROUND(B5/B6,0)</f>
+        <v/>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>社長案（売上6,300万円・粗利2,200万円・販管費2,000万円・経常利益170万円）</t>
+          <t>粗利÷粗利率で計算（2026-10-01検討案：粗利2,150万円・粗利率35%）</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>年間予算粗利</t>
+          <t>年間予算粗利（税抜）</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>22000000</v>
+        <v>21500000</v>
       </c>
     </row>
     <row r="6">
@@ -558,9 +559,8 @@
           <t>予算粗利率</t>
         </is>
       </c>
-      <c r="B6" s="12">
-        <f>B5/B4</f>
-        <v/>
+      <c r="B6" s="6" t="n">
+        <v>0.35</v>
       </c>
     </row>
     <row r="7">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>51000</v>
+        <v>50000</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
@@ -1476,7 +1476,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>考え方：第1段階（月3万円・年36万円）は予算達成時の経常利益の約半分。第2段階は、105%達成で増える利益（年約88万円）の約3割を上乗せした額（月5.1万円・年61万円）。</t>
+          <t>考え方：第1段階（月3万円・年36万円）は予算達成時の経常利益の約半分。第2段階は月5万円・年60万円（105%達成で増える利益 年約86万円の一部を上乗せ）。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Other part-timers: 2 people (workbook and simulator)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H5mKNMdAhueiuoU89hTodu
</commit_message>
<xml_diff>
--- a/excel/Weekends_予算と報奨金_まとめ.xlsx
+++ b/excel/Weekends_予算と報奨金_まとめ.xlsx
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>10</v>
@@ -2009,7 +2009,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>3000</v>

</xml_diff>